<commit_message>
Add VLAN configurations for Lima, Ica, La Libertad, Puno, and Huánuco to the final report and update addressing scheme script
</commit_message>
<xml_diff>
--- a/LIMA-ESQUEMA-DIRECCIONAMIENTO-IA.xlsx
+++ b/LIMA-ESQUEMA-DIRECCIONAMIENTO-IA.xlsx
@@ -214,7 +214,7 @@
         </is>
       </c>
       <c r="E8" s="6">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F8" s="6">
         <v>8</v>
@@ -271,7 +271,7 @@
         </is>
       </c>
       <c r="E9" s="6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" s="6">
         <v>7</v>
@@ -328,7 +328,7 @@
         </is>
       </c>
       <c r="E10" s="6">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="F10" s="6">
         <v>6</v>
@@ -385,7 +385,7 @@
         </is>
       </c>
       <c r="E11" s="6">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="F11" s="6">
         <v>6</v>
@@ -442,7 +442,7 @@
         </is>
       </c>
       <c r="E12" s="6">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="F12" s="6">
         <v>6</v>
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="E13" s="6">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F13" s="6">
         <v>6</v>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="E14" s="6">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="F14" s="6">
         <v>5</v>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="E16" s="6">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="F16" s="6">
         <v>4</v>

</xml_diff>